<commit_message>
Mise à jour du document et modification des images
</commit_message>
<xml_diff>
--- a/projet/backend/data/reseau_kadutu.xlsx
+++ b/projet/backend/data/reseau_kadutu.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projet\BAC3\projet\backend\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02C8929A-7994-48CB-873B-EF0498A6D73C}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{485B1E65-6E7A-4E56-8ACA-5F1324DB5A1D}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12650" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12650" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="NOEUDS" sheetId="1" r:id="rId1"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="142" uniqueCount="69">
   <si>
     <t>P001</t>
   </si>
@@ -225,13 +225,25 @@
   </si>
   <si>
     <t>Nkafu</t>
+  </si>
+  <si>
+    <t>N006</t>
+  </si>
+  <si>
+    <t>N007</t>
+  </si>
+  <si>
+    <t>P005</t>
+  </si>
+  <si>
+    <t>Conduite secondaire 3</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -243,6 +255,14 @@
       <b/>
       <sz val="11"/>
       <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -274,7 +294,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -287,6 +307,21 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -568,7 +603,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="5" width="32.1796875" style="3" customWidth="1"/>
@@ -676,6 +711,40 @@
         <v>28.844999999999999</v>
       </c>
     </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A7" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D7" s="3">
+        <v>-2.5299999999999998</v>
+      </c>
+      <c r="E7" s="3">
+        <v>28.859000000000002</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A8" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D8" s="3">
+        <v>-2.4830000000000001</v>
+      </c>
+      <c r="E8" s="3">
+        <v>28.846</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
@@ -684,7 +753,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E4009069-E252-4C8B-B3AB-54A46E3E8FB3}">
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="7" width="23.26953125" style="3" customWidth="1"/>
@@ -805,6 +874,32 @@
         <v>28</v>
       </c>
     </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A6" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="E6" s="3">
+        <v>250</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="B7" s="5"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -812,135 +907,249 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0A1DADC7-EDB3-4AB5-A67A-8C1AA036A75D}">
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D17"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="4" width="37.453125" style="3" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="8" t="s">
         <v>40</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="8" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A2" s="1" t="s">
+      <c r="A2" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="1">
+      <c r="B2" s="7">
         <v>1</v>
       </c>
-      <c r="C2" s="1">
+      <c r="C2" s="7">
         <v>-2.4849999999999999</v>
       </c>
-      <c r="D2" s="1">
+      <c r="D2" s="7">
         <v>28.835000000000001</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A3" s="1" t="s">
+      <c r="A3" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="1">
+      <c r="B3" s="7">
         <v>2</v>
       </c>
-      <c r="C3" s="1">
+      <c r="C3" s="7">
+        <v>-2.5</v>
+      </c>
+      <c r="D3" s="7">
+        <v>28.858000000000001</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A4" s="9" t="s">
+        <v>0</v>
+      </c>
+      <c r="B4" s="7">
+        <v>3</v>
+      </c>
+      <c r="C4" s="7">
+        <v>-2.5</v>
+      </c>
+      <c r="D4" s="7">
+        <v>28.858000000000001</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A5" s="9" t="s">
+        <v>0</v>
+      </c>
+      <c r="B5" s="7">
+        <v>4</v>
+      </c>
+      <c r="C5" s="7">
         <v>-2.4849999999999999</v>
       </c>
-      <c r="D3" s="1">
+      <c r="D5" s="7">
         <v>28.854800000000001</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A4" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B4" s="1">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A6" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="B6" s="7">
+        <v>1</v>
+      </c>
+      <c r="C6" s="7">
+        <v>-2.4849999999999999</v>
+      </c>
+      <c r="D6" s="7">
+        <v>28.854800000000001</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A7" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="B7" s="7">
+        <v>2</v>
+      </c>
+      <c r="C7" s="7">
+        <v>-2.5</v>
+      </c>
+      <c r="D7" s="7">
+        <v>28.858000000000001</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A8" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="B8" s="7">
         <v>3</v>
       </c>
-      <c r="C4" s="1">
+      <c r="C8" s="7">
         <v>-2.5</v>
       </c>
-      <c r="D4" s="1">
+      <c r="D8" s="7">
         <v>28.858000000000001</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A5" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B5" s="1">
-        <v>4</v>
-      </c>
-      <c r="C5" s="1">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A9" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="B9" s="7">
+        <v>1</v>
+      </c>
+      <c r="C9" s="7">
+        <v>-2.5</v>
+      </c>
+      <c r="D9" s="7">
+        <v>28.858000000000001</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A10" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="B10" s="7">
+        <v>2</v>
+      </c>
+      <c r="C10" s="7">
+        <v>-2.5</v>
+      </c>
+      <c r="D10" s="7">
+        <v>28.858000000000001</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A11" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="B11" s="7">
+        <v>3</v>
+      </c>
+      <c r="C11" s="7">
         <v>-2.52</v>
       </c>
-      <c r="D5" s="1">
+      <c r="D11" s="7">
         <v>28.855</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A6" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="B6" s="1">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A12" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="B12" s="7">
         <v>1</v>
       </c>
-      <c r="C6" s="1">
+      <c r="C12" s="7">
+        <v>-2.52</v>
+      </c>
+      <c r="D12" s="7">
+        <v>28.855</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A13" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="B13" s="7">
+        <v>2</v>
+      </c>
+      <c r="C13" s="7">
+        <v>-2.5</v>
+      </c>
+      <c r="D13" s="7">
+        <v>28.858000000000001</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A14" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="B14" s="7">
+        <v>3</v>
+      </c>
+      <c r="C14" s="7">
         <v>-2.5375000000000001</v>
       </c>
-      <c r="D6" s="1">
+      <c r="D14" s="7">
         <v>28.844999999999999</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A7" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="B7" s="1">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A15" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="B15" s="7">
+        <v>1</v>
+      </c>
+      <c r="C15" s="7">
+        <v>-2.5375000000000001</v>
+      </c>
+      <c r="D15" s="7">
+        <v>28.844999999999999</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A16" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="B16" s="7">
         <v>2</v>
       </c>
-      <c r="C7" s="1">
-        <v>-2.4849999999999999</v>
-      </c>
-      <c r="D7" s="1">
-        <v>28.835000000000001</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A8" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="B8" s="1">
+      <c r="C16" s="7">
+        <v>-2.5</v>
+      </c>
+      <c r="D16" s="7">
+        <v>28.858000000000001</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A17" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="B17" s="7">
         <v>3</v>
       </c>
-      <c r="C8" s="1">
-        <v>-2.4849999999999999</v>
-      </c>
-      <c r="D8" s="1">
-        <v>28.854800000000001</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="C9" s="1"/>
-      <c r="D9" s="1"/>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="C10" s="1"/>
-      <c r="D10" s="1"/>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="C11" s="1"/>
-      <c r="D11" s="1"/>
+      <c r="C17" s="7">
+        <v>-2.5299999999999998</v>
+      </c>
+      <c r="D17" s="7">
+        <v>28.859000000000002</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>